<commit_message>
P2 #1: Sweep remaining XP display sites to formatXP() helper
Migrated 14 additional sites in App.js from `.toLocaleString() + " XP"` to
the canonical formatXP() helper introduced in #59. Sites covered:
- Quest complete toast (1732)
- Plan complete toast (2728)
- XP flash widget (3199)
- Workout-tag chip in upcoming list (4715)
- Workout builder total (5159)
- Superset accordion total (5211)
- Quest reward badge (6442)
- Log group meta + log group XP (6527, 6594, 6688)
- Workout/plan delete confirmation dialogs (6610, 6704)
- Battle Record header (6730)
- Friends feed XP (6961)
- Workout completion sub (9512)

Sites left as `.toLocaleString()` are genuinely number-only — the "XP" label
is supplied by a sibling span (e.g. `eff-weight-lbl: "XP earned"`,
`combat-chip-lbl: "Total XP"`, `xp-proj-value` chips, "Est. XP:" prefix).

Regenerated Aurisar_Audit_Report.xlsx to reflect the lower remaining count.

Verification: npm run build passes.
</commit_message>
<xml_diff>
--- a/Aurisar_Audit_Report.xlsx
+++ b/Aurisar_Audit_Report.xlsx
@@ -552,7 +552,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
@@ -567,7 +567,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>

</xml_diff>